<commit_message>
fix(sheets): 민요 검수 xlsx ○ 기호 제거
</commit_message>
<xml_diff>
--- a/sheets/민요/검수/강강술래.xlsx
+++ b/sheets/민요/검수/강강술래.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="143">
   <si>
     <t xml:space="preserve">강강술래</t>
   </si>
@@ -727,6 +727,9 @@
     <t xml:space="preserve">南
 –
 △ </t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
   </si>
 </sst>
 </file>
@@ -1903,10 +1906,10 @@
         <v>4</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="I17" s="4"/>
       <c r="J17" s="3"/>

</xml_diff>